<commit_message>
[Nairne] Apr 2026 corrections: +$20K JJNA accrual, consolidate positions
- JJNA April beginning balance bumped by $20K (per upcoming end-of-month
  statement) — total carryforward now $40K + $8M April call = $8,040,000
- Total LP base $8,548,472, gross profit recomputed to $487,262.90
- GP distribution to Innovations: $119,866.67 (Nairne $71,920.00 /
  Alec $47,347.34 / Chris $599.33)
- Investment Positions: with JJNA's tranche formally closed, all working
  capital ($8,828,160.91) now sits in the Armada Innovations trading
  sleeve. Removed Undeployed Capital line — May investors haven't funded
  yet, so no undeployed capital at April month-end.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/april-2026-allocation.xlsx
+++ b/armada-innovations/data/april-2026-allocation.xlsx
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>March 31 PCAS ending balance</t>
+          <t>March 31 PCAS ending balance + $20K additional accrual (per April end-of-month statement, pending)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[Nairne] Apr 2026: revert JJNA $20K addition (was double-count)
The PCAS confirms JJNA's March-end balance is $20K total, not $40K.
The 'additional $20K' instruction was a misread — that $20K was already
captured in JJNA's March accrual carryforward.

Reverts April math to: gross $486,122.90 on $8,528,472 base, GP cut
$119,586.23 (Nairne $71,751.74 / Alec $47,236.56 / Chris $597.93).

Investment Positions remain consolidated under the Armada Innovations
trading sleeve (no Undeployed Capital line).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/april-2026-allocation.xlsx
+++ b/armada-innovations/data/april-2026-allocation.xlsx
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>March 31 PCAS ending balance + $20K additional accrual (per April end-of-month statement, pending)</t>
+          <t>March 31 PCAS ending balance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[Nairne] Add Brokerage Attribution tab — full Mar→Apr→May flow
New tab in april-2026-allocation.xlsx showing the chronological flow of
every dollar in the brokerage account across all parties:

- Capital contributed (lifetime)
- Mar 31 balance (= Apr 1 beginning)
- + April activity (LP cuts, TQ fee, GP distribution)
- + May wire (new investors received in advance)
- = Current balance (May 1, 2026)

Tie-out: $8,532,056.10 + $486,122.90 + $1,499,728.00 = $10,517,907.00
Brokerage actual: $10,519,780.00 → leftover $1,873 (≈1 day fund growth).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/april-2026-allocation.xlsx
+++ b/armada-innovations/data/april-2026-allocation.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April 2026 Allocation" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Who Gets What" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brokerage Attribution" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red](&quot;$&quot;#,##0.00)"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +50,14 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="8">
@@ -115,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,6 +164,15 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1357,4 +1375,279 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>Brokerage Account Attribution Flow — May 1, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Where every dollar in the brokerage came from and where it sits today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="B4" s="38" t="inlineStr">
+        <is>
+          <t>Capital Contributed</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>Mar 31 Balance (= Apr 1 Beg)</t>
+        </is>
+      </c>
+      <c r="D4" s="38" t="inlineStr">
+        <is>
+          <t>+ Apr Activity (net of fees)</t>
+        </is>
+      </c>
+      <c r="E4" s="38" t="inlineStr">
+        <is>
+          <t>+ May Wire (advance)</t>
+        </is>
+      </c>
+      <c r="F4" s="38" t="inlineStr">
+        <is>
+          <t>Current Balance (May 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Bliss Investments LLC</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>508472</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>16636.19</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>525108.1899999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>JJNA, LLC</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>8020000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>262398.36</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>8282398.36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>New May Investors</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>1499728</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>1499728</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>1499728</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>TruQuant (accrued payable)</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>87502.12</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>87502.12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Innovations GP (accrued)</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>3720</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>119586.23</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>123306.23</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Bank-fee cash carry</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="41" t="n">
+        <v>-135.9</v>
+      </c>
+      <c r="D10" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="41" t="n">
+        <v>-135.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL ATTRIBUTED</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>SUM(B5:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="13">
+        <f>SUM(C5:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="13">
+        <f>SUM(E5:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="13">
+        <f>SUM(F5:F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Brokerage actual (live)</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="42" t="n"/>
+      <c r="D12" s="42" t="n"/>
+      <c r="E12" s="42" t="n"/>
+      <c r="F12" s="16" t="n">
+        <v>10519780</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>LEFTOVER (≈1 day fund growth)</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="42" t="n"/>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="16">
+        <f>F12-F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>Tie-out:  Mar 31 base + Apr activity + May advance = Current Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>C11&amp;" + "&amp;D11&amp;" + "&amp;E11&amp;" = "&amp;F11</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[Nairne] Brokerage attribution: account for GP monthly sweep
Innovations LLC sweeps its distribution out at the start of each month,
so during April the GP had $0 in the brokerage:
- Mar 31 GP balance shows $0 (Mar's $3,720 was swept on Apr 1)
- Today's GP-in-brokerage = $119,586.23 (April accrual, will sweep May 1)

This drops total attributed by $3,720 to $10,514,187 → leftover $5,593
(~3 days of fund growth between Apr 30 and May 1).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/april-2026-allocation.xlsx
+++ b/armada-innovations/data/april-2026-allocation.xlsx
@@ -1383,10 +1383,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
@@ -1404,249 +1404,266 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Where every dollar in the brokerage came from and where it sits today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
+          <t>GP rule: Innovations LLC sweeps its monthly distribution out at the start of the next month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>→ Mar GP $3,720 paid out Apr 1 (Innovations had $0 in fund during April).  Apr GP $119,586.23 sits in brokerage today, will sweep at start of May.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Party</t>
         </is>
       </c>
-      <c r="B4" s="38" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>Capital Contributed</t>
         </is>
       </c>
-      <c r="C4" s="38" t="inlineStr">
-        <is>
-          <t>Mar 31 Balance (= Apr 1 Beg)</t>
-        </is>
-      </c>
-      <c r="D4" s="38" t="inlineStr">
-        <is>
-          <t>+ Apr Activity (net of fees)</t>
-        </is>
-      </c>
-      <c r="E4" s="38" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>Mar 31 Bal (= Apr 1 Beg)</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>+ Apr Activity (net)</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
         <is>
           <t>+ May Wire (advance)</t>
         </is>
       </c>
-      <c r="F4" s="38" t="inlineStr">
+      <c r="F5" s="38" t="inlineStr">
         <is>
           <t>Current Balance (May 1)</t>
         </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>Bliss Investments LLC</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C5" s="9" t="n">
-        <v>508472</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>16636.19</v>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>525108.1899999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="30" t="inlineStr">
         <is>
-          <t>JJNA, LLC</t>
+          <t>Bliss Investments LLC</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>8000000</v>
+        <v>500000</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>8020000</v>
+        <v>508472</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>262398.36</v>
+        <v>16636.19</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
+        <v>525108.1899999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>JJNA, LLC</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>8020000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>262398.36</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>8282398.36</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>New May Investors</t>
         </is>
       </c>
-      <c r="B7" s="40" t="n">
+      <c r="B8" s="40" t="n">
         <v>1499728</v>
       </c>
-      <c r="C7" s="40" t="n">
+      <c r="C8" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="40" t="n">
+      <c r="D8" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E8" s="40" t="n">
         <v>1499728</v>
       </c>
-      <c r="F7" s="40" t="n">
+      <c r="F8" s="40" t="n">
         <v>1499728</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>TruQuant (accrued payable)</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D9" s="19" t="n">
         <v>87502.12</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F9" s="19" t="n">
         <v>87502.12</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>Innovations GP (accrued)</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n">
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Innovations GP (Apr accrual, awaiting May sweep)</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="25" t="n">
-        <v>3720</v>
-      </c>
-      <c r="D9" s="25" t="n">
+      <c r="C10" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25" t="n">
         <v>119586.23</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E10" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="25" t="n">
-        <v>123306.23</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="F10" s="25" t="n">
+        <v>119586.23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Bank-fee cash carry</t>
         </is>
       </c>
-      <c r="B10" s="41" t="n">
+      <c r="B11" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="41" t="n">
+      <c r="C11" s="41" t="n">
         <v>-135.9</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D11" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="41" t="n">
+      <c r="E11" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="41" t="n">
+      <c r="F11" s="41" t="n">
         <v>-135.9</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>TOTAL ATTRIBUTED</t>
         </is>
       </c>
-      <c r="B11" s="13">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="13">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="13">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="13">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="13">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Brokerage actual (live)</t>
-        </is>
-      </c>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="42" t="n"/>
-      <c r="F12" s="16" t="n">
-        <v>10519780</v>
+      <c r="B12" s="13">
+        <f>SUM(B6:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="13">
+        <f>SUM(C6:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>SUM(D6:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="13">
+        <f>SUM(E6:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="13">
+        <f>SUM(F6:F11)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>LEFTOVER (≈1 day fund growth)</t>
+          <t>Brokerage actual (live)</t>
         </is>
       </c>
       <c r="B13" s="42" t="n"/>
       <c r="C13" s="42" t="n"/>
       <c r="D13" s="42" t="n"/>
       <c r="E13" s="42" t="n"/>
-      <c r="F13" s="16">
-        <f>F12-F11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="43" t="inlineStr">
-        <is>
-          <t>Tie-out:  Mar 31 base + Apr activity + May advance = Current Balance</t>
-        </is>
+      <c r="F13" s="16" t="n">
+        <v>10519780</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>LEFTOVER (≈3 days fund growth)</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="42" t="n"/>
+      <c r="E14" s="42" t="n"/>
+      <c r="F14" s="16">
+        <f>F13-F12</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <f>C11&amp;" + "&amp;D11&amp;" + "&amp;E11&amp;" = "&amp;F11</f>
-        <v/>
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>Tie-out: Mar 31 base + Apr activity + May advance = Current Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>Already paid out (NOT in current brokerage):</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Mar GP distribution $3,720 → swept Apr 1 to Innovations bank (Nairne $2,232 / Alec $1,469.40 / Chris $18.60)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>